<commit_message>
add: Cambio Excel carga facturas para poder guardar correctamente la fecha, y el tipo de cliente proveedor, ademas se realizo el cambio en Compra Impuestos quitando la referencia de Tb_Sustentos por un enumerador y borrando la tabla de sustentos, en codigos compra impuestos se realizo lo mismo quitando la referencia a codigo sustento y colocando un enumerador.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/CargarFacturas.xlsx
+++ b/api/src/main/resources/CargarFacturas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28EC3A0-251C-4DF7-A2AF-EEBE1195EB96}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6553A1-7F1F-46FE-A905-509680BE20D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{D556B04B-A296-4224-AEE4-E6FD1C8884D2}"/>
   </bookViews>
@@ -87,12 +87,6 @@
     <t>Descuento</t>
   </si>
   <si>
-    <t>Codigo IVA</t>
-  </si>
-  <si>
-    <t>PORCENTAJE IVA</t>
-  </si>
-  <si>
     <t>Caja-Banco</t>
   </si>
   <si>
@@ -267,10 +261,16 @@
     <t>PAIS</t>
   </si>
   <si>
-    <t>01/04/2024</t>
-  </si>
-  <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>Codigo Impuesto</t>
+  </si>
+  <si>
+    <t>Codigo Porcentaje</t>
+  </si>
+  <si>
+    <t>19/05/2026</t>
   </si>
 </sst>
 </file>
@@ -691,6 +691,8 @@
     <col min="5" max="5" width="17.28515625" customWidth="1"/>
     <col min="6" max="6" width="22.85546875" customWidth="1"/>
     <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
+    <col min="22" max="22" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.25">
@@ -755,110 +757,112 @@
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="AB1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AP1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="I2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="8" t="s">
+      <c r="J2" s="9" t="s">
         <v>40</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="N2" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" s="10" t="s">
-        <v>45</v>
       </c>
       <c r="O2" s="10"/>
       <c r="P2" s="10"/>
@@ -873,16 +877,16 @@
         <v>2</v>
       </c>
       <c r="U2" s="12">
+        <v>2</v>
+      </c>
+      <c r="V2" s="12">
         <v>4</v>
       </c>
-      <c r="V2" s="12">
-        <v>15</v>
-      </c>
       <c r="W2" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X2" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Y2" s="9">
         <v>55565556</v>
@@ -892,7 +896,7 @@
       </c>
       <c r="AA2" s="9"/>
       <c r="AB2" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AC2" s="9"/>
       <c r="AD2" s="9"/>
@@ -911,41 +915,43 @@
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="L3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="M3" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="M3" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -961,16 +967,16 @@
         <v>0</v>
       </c>
       <c r="U3" s="12">
+        <v>2</v>
+      </c>
+      <c r="V3" s="12">
         <v>4</v>
       </c>
-      <c r="V3" s="12">
-        <v>15</v>
-      </c>
       <c r="W3" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="Y3" s="9">
         <v>55565556</v>
@@ -997,41 +1003,43 @@
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="13" t="s">
+      <c r="I4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L4" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N4" s="10"/>
       <c r="O4" s="10"/>
@@ -1047,16 +1055,16 @@
         <v>5</v>
       </c>
       <c r="U4" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V4" s="12">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="Y4" s="9">
         <v>445244</v>
@@ -1083,41 +1091,43 @@
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G5" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="13" t="s">
+      <c r="I5" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>62</v>
-      </c>
       <c r="J5" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N5" s="10"/>
       <c r="O5" s="10"/>
@@ -1133,16 +1143,16 @@
         <v>8</v>
       </c>
       <c r="U5" s="12">
+        <v>2</v>
+      </c>
+      <c r="V5" s="12">
         <v>4</v>
       </c>
-      <c r="V5" s="12">
-        <v>15</v>
-      </c>
       <c r="W5" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="X5" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="Y5" s="9"/>
       <c r="Z5" s="7">
@@ -1167,41 +1177,43 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="13" t="s">
+      <c r="I6" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F6" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="8" t="s">
+      <c r="J6" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="K6" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>70</v>
-      </c>
       <c r="L6" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
@@ -1217,16 +1229,16 @@
         <v>2</v>
       </c>
       <c r="U6" s="12">
+        <v>2</v>
+      </c>
+      <c r="V6" s="12">
         <v>4</v>
       </c>
-      <c r="V6" s="12">
-        <v>15</v>
-      </c>
       <c r="W6" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="Y6" s="9">
         <v>66445</v>
@@ -1253,41 +1265,43 @@
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="8" t="s">
+      <c r="J7" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="K7" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="J7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L7" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
@@ -1303,16 +1317,16 @@
         <v>2</v>
       </c>
       <c r="U7" s="12">
+        <v>2</v>
+      </c>
+      <c r="V7" s="12">
         <v>4</v>
       </c>
-      <c r="V7" s="12">
-        <v>15</v>
-      </c>
       <c r="W7" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X7" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="Y7" s="9">
         <v>54455477</v>
@@ -1339,41 +1353,43 @@
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E8" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="8" t="s">
+      <c r="J8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="K8" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K8" s="14" t="s">
-        <v>57</v>
-      </c>
       <c r="L8" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
@@ -1389,16 +1405,16 @@
         <v>2</v>
       </c>
       <c r="U8" s="12">
+        <v>2</v>
+      </c>
+      <c r="V8" s="12">
         <v>4</v>
       </c>
-      <c r="V8" s="12">
-        <v>15</v>
-      </c>
       <c r="W8" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="X8" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Y8" s="9"/>
       <c r="Z8" s="7"/>
@@ -1423,41 +1439,43 @@
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E9" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="8" t="s">
+      <c r="J9" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="K9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L9" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
@@ -1473,16 +1491,16 @@
         <v>2</v>
       </c>
       <c r="U9" s="12">
+        <v>2</v>
+      </c>
+      <c r="V9" s="12">
         <v>4</v>
       </c>
-      <c r="V9" s="12">
-        <v>15</v>
-      </c>
       <c r="W9" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="X9" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Y9" s="9"/>
       <c r="Z9" s="7"/>
@@ -1507,39 +1525,39 @@
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B10" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>77</v>
-      </c>
       <c r="F10" s="16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G10" s="13" t="b">
         <v>1</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
       <c r="L10" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
@@ -1555,16 +1573,16 @@
         <v>2</v>
       </c>
       <c r="U10" s="12">
+        <v>2</v>
+      </c>
+      <c r="V10" s="12">
         <v>4</v>
       </c>
-      <c r="V10" s="12">
-        <v>15</v>
-      </c>
       <c r="W10" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="X10" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Y10" s="9"/>
       <c r="Z10" s="7"/>

</xml_diff>